<commit_message>
Updated JPN_grids_kan model - 2026-05-01 19:04
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01EB8F7F-9995-4A63-B2DB-E83CE843CB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7196D768-B727-4802-AFE3-76B362552823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1288" uniqueCount="688">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -349,1729 +349,1759 @@
     <t>t_pos_andor</t>
   </si>
   <si>
-    <t>p_w66098469</t>
-  </si>
-  <si>
-    <t>e_w66098469*</t>
+    <t>p_w66098469-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w66098469-500_JPN*</t>
   </si>
   <si>
     <t>OR</t>
   </si>
   <si>
-    <t>p_w87538349</t>
-  </si>
-  <si>
-    <t>e_w87538349*</t>
-  </si>
-  <si>
-    <t>p_w102958903</t>
-  </si>
-  <si>
-    <t>e_w102958903*</t>
-  </si>
-  <si>
-    <t>p_w104173570</t>
-  </si>
-  <si>
-    <t>e_w104173570*</t>
-  </si>
-  <si>
-    <t>p_w104391636</t>
-  </si>
-  <si>
-    <t>e_w104391636*</t>
-  </si>
-  <si>
-    <t>p_w104530060</t>
-  </si>
-  <si>
-    <t>e_w104530060*</t>
-  </si>
-  <si>
-    <t>p_w105298089</t>
-  </si>
-  <si>
-    <t>e_w105298089*</t>
-  </si>
-  <si>
-    <t>p_w106076988</t>
-  </si>
-  <si>
-    <t>e_w106076988*</t>
-  </si>
-  <si>
-    <t>p_w106309481</t>
-  </si>
-  <si>
-    <t>e_w106309481*</t>
-  </si>
-  <si>
-    <t>p_w109834508</t>
-  </si>
-  <si>
-    <t>e_w109834508*</t>
-  </si>
-  <si>
-    <t>p_w109850439</t>
-  </si>
-  <si>
-    <t>e_w109850439*</t>
-  </si>
-  <si>
-    <t>p_w110682956</t>
-  </si>
-  <si>
-    <t>e_w110682956*</t>
-  </si>
-  <si>
-    <t>p_w116559939</t>
-  </si>
-  <si>
-    <t>e_w116559939*</t>
-  </si>
-  <si>
-    <t>p_w128581912</t>
-  </si>
-  <si>
-    <t>e_w128581912*</t>
-  </si>
-  <si>
-    <t>p_w132913106</t>
-  </si>
-  <si>
-    <t>e_w132913106*</t>
-  </si>
-  <si>
-    <t>p_w133641619</t>
-  </si>
-  <si>
-    <t>e_w133641619*</t>
-  </si>
-  <si>
-    <t>p_w133644487</t>
-  </si>
-  <si>
-    <t>e_w133644487*</t>
-  </si>
-  <si>
-    <t>p_w142662111</t>
-  </si>
-  <si>
-    <t>e_w142662111*</t>
-  </si>
-  <si>
-    <t>p_w145079972</t>
-  </si>
-  <si>
-    <t>e_w145079972*</t>
-  </si>
-  <si>
-    <t>p_w149843487</t>
-  </si>
-  <si>
-    <t>e_w149843487*</t>
-  </si>
-  <si>
-    <t>p_w150035494</t>
-  </si>
-  <si>
-    <t>e_w150035494*</t>
-  </si>
-  <si>
-    <t>p_w150065045</t>
-  </si>
-  <si>
-    <t>e_w150065045*</t>
-  </si>
-  <si>
-    <t>p_w151379730</t>
-  </si>
-  <si>
-    <t>e_w151379730*</t>
-  </si>
-  <si>
-    <t>p_w156208858</t>
-  </si>
-  <si>
-    <t>e_w156208858*</t>
-  </si>
-  <si>
-    <t>p_w161727149</t>
-  </si>
-  <si>
-    <t>e_w161727149*</t>
-  </si>
-  <si>
-    <t>p_w161870227</t>
-  </si>
-  <si>
-    <t>e_w161870227*</t>
-  </si>
-  <si>
-    <t>p_w161946849</t>
-  </si>
-  <si>
-    <t>e_w161946849*</t>
-  </si>
-  <si>
-    <t>p_w168727982</t>
-  </si>
-  <si>
-    <t>e_w168727982*</t>
-  </si>
-  <si>
-    <t>p_w168839127</t>
-  </si>
-  <si>
-    <t>e_w168839127*</t>
-  </si>
-  <si>
-    <t>p_w168857610</t>
-  </si>
-  <si>
-    <t>e_w168857610*</t>
-  </si>
-  <si>
-    <t>p_w169031921</t>
-  </si>
-  <si>
-    <t>e_w169031921*</t>
-  </si>
-  <si>
-    <t>p_w169031998</t>
-  </si>
-  <si>
-    <t>e_w169031998*</t>
-  </si>
-  <si>
-    <t>p_w169122898</t>
-  </si>
-  <si>
-    <t>e_w169122898*</t>
-  </si>
-  <si>
-    <t>p_w169249243</t>
-  </si>
-  <si>
-    <t>e_w169249243*</t>
-  </si>
-  <si>
-    <t>p_w256682313</t>
-  </si>
-  <si>
-    <t>e_w256682313*</t>
-  </si>
-  <si>
-    <t>p_w169359724</t>
-  </si>
-  <si>
-    <t>e_w169359724*</t>
-  </si>
-  <si>
-    <t>p_w169963227</t>
-  </si>
-  <si>
-    <t>e_w169963227*</t>
-  </si>
-  <si>
-    <t>p_w170247312</t>
-  </si>
-  <si>
-    <t>e_w170247312*</t>
-  </si>
-  <si>
-    <t>p_w170366035</t>
-  </si>
-  <si>
-    <t>e_w170366035*</t>
-  </si>
-  <si>
-    <t>p_w170537514</t>
-  </si>
-  <si>
-    <t>e_w170537514*</t>
-  </si>
-  <si>
-    <t>p_w170568495</t>
-  </si>
-  <si>
-    <t>e_w170568495*</t>
-  </si>
-  <si>
-    <t>p_w170589736</t>
-  </si>
-  <si>
-    <t>e_w170589736*</t>
-  </si>
-  <si>
-    <t>p_w170605907</t>
-  </si>
-  <si>
-    <t>e_w170605907*</t>
-  </si>
-  <si>
-    <t>p_w170850727</t>
-  </si>
-  <si>
-    <t>e_w170850727*</t>
-  </si>
-  <si>
-    <t>p_w170974371</t>
-  </si>
-  <si>
-    <t>e_w170974371*</t>
-  </si>
-  <si>
-    <t>p_w171066843</t>
-  </si>
-  <si>
-    <t>e_w171066843*</t>
-  </si>
-  <si>
-    <t>p_w172144358</t>
-  </si>
-  <si>
-    <t>e_w172144358*</t>
-  </si>
-  <si>
-    <t>p_w172601929</t>
-  </si>
-  <si>
-    <t>e_w172601929*</t>
-  </si>
-  <si>
-    <t>p_w172907196</t>
-  </si>
-  <si>
-    <t>e_w172907196*</t>
-  </si>
-  <si>
-    <t>p_w174636874</t>
-  </si>
-  <si>
-    <t>e_w174636874*</t>
-  </si>
-  <si>
-    <t>p_w185029969</t>
-  </si>
-  <si>
-    <t>e_w185029969*</t>
-  </si>
-  <si>
-    <t>p_w186510275</t>
-  </si>
-  <si>
-    <t>e_w186510275*</t>
-  </si>
-  <si>
-    <t>p_w187988970</t>
-  </si>
-  <si>
-    <t>e_w187988970*</t>
-  </si>
-  <si>
-    <t>p_w190769051</t>
-  </si>
-  <si>
-    <t>e_w190769051*</t>
-  </si>
-  <si>
-    <t>p_w193544791</t>
-  </si>
-  <si>
-    <t>e_w193544791*</t>
-  </si>
-  <si>
-    <t>p_w195615141</t>
-  </si>
-  <si>
-    <t>e_w195615141*</t>
-  </si>
-  <si>
-    <t>p_w201293312</t>
-  </si>
-  <si>
-    <t>e_w201293312*</t>
-  </si>
-  <si>
-    <t>p_w204258596</t>
-  </si>
-  <si>
-    <t>e_w204258596*</t>
-  </si>
-  <si>
-    <t>p_w209429410</t>
-  </si>
-  <si>
-    <t>e_w209429410*</t>
-  </si>
-  <si>
-    <t>p_w209726348</t>
-  </si>
-  <si>
-    <t>e_w209726348*</t>
-  </si>
-  <si>
-    <t>p_w210090094</t>
-  </si>
-  <si>
-    <t>e_w210090094*</t>
-  </si>
-  <si>
-    <t>p_w211412000</t>
-  </si>
-  <si>
-    <t>e_w211412000*</t>
-  </si>
-  <si>
-    <t>p_w215451416</t>
-  </si>
-  <si>
-    <t>e_w215451416*</t>
-  </si>
-  <si>
-    <t>p_w216502300</t>
-  </si>
-  <si>
-    <t>e_w216502300*</t>
-  </si>
-  <si>
-    <t>p_w216778426</t>
-  </si>
-  <si>
-    <t>e_w216778426*</t>
-  </si>
-  <si>
-    <t>p_w216953915</t>
-  </si>
-  <si>
-    <t>e_w216953915*</t>
-  </si>
-  <si>
-    <t>p_w216956620</t>
-  </si>
-  <si>
-    <t>e_w216956620*</t>
-  </si>
-  <si>
-    <t>p_w241822621</t>
-  </si>
-  <si>
-    <t>e_w241822621*</t>
-  </si>
-  <si>
-    <t>p_w241822623</t>
-  </si>
-  <si>
-    <t>e_w241822623*</t>
-  </si>
-  <si>
-    <t>p_w241822631</t>
-  </si>
-  <si>
-    <t>e_w241822631*</t>
-  </si>
-  <si>
-    <t>p_w241828221</t>
-  </si>
-  <si>
-    <t>e_w241828221*</t>
-  </si>
-  <si>
-    <t>p_w242103481</t>
-  </si>
-  <si>
-    <t>e_w242103481*</t>
-  </si>
-  <si>
-    <t>p_w242103532</t>
-  </si>
-  <si>
-    <t>e_w242103532*</t>
-  </si>
-  <si>
-    <t>p_w242253500</t>
-  </si>
-  <si>
-    <t>e_w242253500*</t>
-  </si>
-  <si>
-    <t>p_w250540807</t>
-  </si>
-  <si>
-    <t>e_w250540807*</t>
-  </si>
-  <si>
-    <t>p_w253566674</t>
-  </si>
-  <si>
-    <t>e_w253566674*</t>
-  </si>
-  <si>
-    <t>p_w291678103</t>
-  </si>
-  <si>
-    <t>e_w291678103*</t>
-  </si>
-  <si>
-    <t>p_w307942220</t>
-  </si>
-  <si>
-    <t>e_w307942220*</t>
-  </si>
-  <si>
-    <t>p_w315434358</t>
-  </si>
-  <si>
-    <t>e_w315434358*</t>
-  </si>
-  <si>
-    <t>p_w315461259</t>
-  </si>
-  <si>
-    <t>e_w315461259*</t>
-  </si>
-  <si>
-    <t>p_w315461272</t>
-  </si>
-  <si>
-    <t>e_w315461272*</t>
-  </si>
-  <si>
-    <t>p_w315618377</t>
-  </si>
-  <si>
-    <t>e_w315618377*</t>
-  </si>
-  <si>
-    <t>p_w315662839</t>
-  </si>
-  <si>
-    <t>e_w315662839*</t>
-  </si>
-  <si>
-    <t>p_w317416612</t>
-  </si>
-  <si>
-    <t>e_w317416612*</t>
-  </si>
-  <si>
-    <t>p_w317511904</t>
-  </si>
-  <si>
-    <t>e_w317511904*</t>
-  </si>
-  <si>
-    <t>p_w320438391</t>
-  </si>
-  <si>
-    <t>e_w320438391*</t>
-  </si>
-  <si>
-    <t>p_w405626236</t>
-  </si>
-  <si>
-    <t>e_w405626236*</t>
-  </si>
-  <si>
-    <t>p_w421647841</t>
-  </si>
-  <si>
-    <t>e_w421647841*</t>
-  </si>
-  <si>
-    <t>p_w459476442</t>
-  </si>
-  <si>
-    <t>e_w459476442*</t>
-  </si>
-  <si>
-    <t>p_w505170104</t>
-  </si>
-  <si>
-    <t>e_w505170104*</t>
-  </si>
-  <si>
-    <t>p_w659138214</t>
-  </si>
-  <si>
-    <t>e_w659138214*</t>
-  </si>
-  <si>
-    <t>p_w714627759</t>
-  </si>
-  <si>
-    <t>e_w714627759*</t>
-  </si>
-  <si>
-    <t>p_w722673849</t>
-  </si>
-  <si>
-    <t>e_w722673849*</t>
-  </si>
-  <si>
-    <t>p_w785319805</t>
-  </si>
-  <si>
-    <t>e_w785319805*</t>
-  </si>
-  <si>
-    <t>p_w832823487</t>
-  </si>
-  <si>
-    <t>e_w832823487*</t>
-  </si>
-  <si>
-    <t>p_w901872431</t>
-  </si>
-  <si>
-    <t>e_w901872431*</t>
-  </si>
-  <si>
-    <t>p_w901872439</t>
-  </si>
-  <si>
-    <t>e_w901872439*</t>
-  </si>
-  <si>
-    <t>p_w1029010255</t>
-  </si>
-  <si>
-    <t>e_w1029010255*</t>
-  </si>
-  <si>
-    <t>p_w975217734</t>
-  </si>
-  <si>
-    <t>e_w975217734*</t>
-  </si>
-  <si>
-    <t>p_w1028554758</t>
-  </si>
-  <si>
-    <t>e_w1028554758*</t>
-  </si>
-  <si>
-    <t>p_w1030329139</t>
-  </si>
-  <si>
-    <t>e_w1030329139*</t>
-  </si>
-  <si>
-    <t>p_w1037299172</t>
-  </si>
-  <si>
-    <t>e_w1037299172*</t>
-  </si>
-  <si>
-    <t>p_w1037516198</t>
-  </si>
-  <si>
-    <t>e_w1037516198*</t>
-  </si>
-  <si>
-    <t>p_w1038584990</t>
-  </si>
-  <si>
-    <t>e_w1038584990*</t>
-  </si>
-  <si>
-    <t>p_r2269992</t>
-  </si>
-  <si>
-    <t>e_r2269992*</t>
-  </si>
-  <si>
-    <t>p_r11529219</t>
-  </si>
-  <si>
-    <t>e_r11529219*</t>
-  </si>
-  <si>
-    <t>p_r11529637</t>
-  </si>
-  <si>
-    <t>e_r11529637*</t>
-  </si>
-  <si>
-    <t>p_r13768299</t>
-  </si>
-  <si>
-    <t>e_r13768299*</t>
-  </si>
-  <si>
-    <t>p_r15580570</t>
-  </si>
-  <si>
-    <t>e_r15580570*</t>
-  </si>
-  <si>
-    <t>p_r17013811</t>
-  </si>
-  <si>
-    <t>e_r17013811*</t>
-  </si>
-  <si>
-    <t>p_JP21</t>
-  </si>
-  <si>
-    <t>e_JP21*</t>
-  </si>
-  <si>
-    <t>p_JP36</t>
-  </si>
-  <si>
-    <t>e_JP36*</t>
-  </si>
-  <si>
-    <t>p_JP28</t>
-  </si>
-  <si>
-    <t>e_JP28*</t>
-  </si>
-  <si>
-    <t>p_JP60</t>
-  </si>
-  <si>
-    <t>e_JP60*</t>
-  </si>
-  <si>
-    <t>p_JP23</t>
-  </si>
-  <si>
-    <t>e_JP23*</t>
-  </si>
-  <si>
-    <t>p_JP95</t>
-  </si>
-  <si>
-    <t>e_JP95*</t>
-  </si>
-  <si>
-    <t>p_JP191</t>
-  </si>
-  <si>
-    <t>e_JP191*</t>
-  </si>
-  <si>
-    <t>p_JP116</t>
-  </si>
-  <si>
-    <t>e_JP116*</t>
-  </si>
-  <si>
-    <t>p_JP156</t>
-  </si>
-  <si>
-    <t>e_JP156*</t>
-  </si>
-  <si>
-    <t>p_JP141</t>
-  </si>
-  <si>
-    <t>e_JP141*</t>
-  </si>
-  <si>
-    <t>p_JP122</t>
-  </si>
-  <si>
-    <t>e_JP122*</t>
-  </si>
-  <si>
-    <t>p_JP178</t>
-  </si>
-  <si>
-    <t>e_JP178*</t>
-  </si>
-  <si>
-    <t>p_JP117</t>
-  </si>
-  <si>
-    <t>e_JP117*</t>
-  </si>
-  <si>
-    <t>p_JP132</t>
-  </si>
-  <si>
-    <t>e_JP132*</t>
-  </si>
-  <si>
-    <t>p_JP269</t>
-  </si>
-  <si>
-    <t>e_JP269*</t>
-  </si>
-  <si>
-    <t>p_JP19</t>
-  </si>
-  <si>
-    <t>e_JP19*</t>
-  </si>
-  <si>
-    <t>p_JP267</t>
-  </si>
-  <si>
-    <t>e_JP267*</t>
-  </si>
-  <si>
-    <t>p_JP102</t>
-  </si>
-  <si>
-    <t>e_JP102*</t>
-  </si>
-  <si>
-    <t>p_JP112</t>
-  </si>
-  <si>
-    <t>e_JP112*</t>
-  </si>
-  <si>
-    <t>p_JP106</t>
-  </si>
-  <si>
-    <t>e_JP106*</t>
-  </si>
-  <si>
-    <t>p_JP96</t>
-  </si>
-  <si>
-    <t>e_JP96*</t>
-  </si>
-  <si>
-    <t>p_JP9</t>
-  </si>
-  <si>
-    <t>e_JP9*</t>
-  </si>
-  <si>
-    <t>p_JP292</t>
-  </si>
-  <si>
-    <t>e_JP292*</t>
-  </si>
-  <si>
-    <t>p_JP294</t>
-  </si>
-  <si>
-    <t>e_JP294*</t>
-  </si>
-  <si>
-    <t>p_JP41</t>
-  </si>
-  <si>
-    <t>e_JP41*</t>
-  </si>
-  <si>
-    <t>p_JP29</t>
-  </si>
-  <si>
-    <t>e_JP29*</t>
-  </si>
-  <si>
-    <t>p_JP37</t>
-  </si>
-  <si>
-    <t>e_JP37*</t>
-  </si>
-  <si>
-    <t>p_JP218</t>
-  </si>
-  <si>
-    <t>e_JP218*</t>
-  </si>
-  <si>
-    <t>p_w242253537</t>
-  </si>
-  <si>
-    <t>e_w242253537*</t>
-  </si>
-  <si>
-    <t>p_JP10</t>
-  </si>
-  <si>
-    <t>e_JP10*</t>
-  </si>
-  <si>
-    <t>p_JP57</t>
-  </si>
-  <si>
-    <t>e_JP57*</t>
-  </si>
-  <si>
-    <t>p_JP30</t>
-  </si>
-  <si>
-    <t>e_JP30*</t>
-  </si>
-  <si>
-    <t>p_JP34</t>
-  </si>
-  <si>
-    <t>e_JP34*</t>
-  </si>
-  <si>
-    <t>p_JP118</t>
-  </si>
-  <si>
-    <t>e_JP118*</t>
-  </si>
-  <si>
-    <t>p_JP119</t>
-  </si>
-  <si>
-    <t>e_JP119*</t>
-  </si>
-  <si>
-    <t>p_JP135</t>
-  </si>
-  <si>
-    <t>e_JP135*</t>
-  </si>
-  <si>
-    <t>p_JP158</t>
-  </si>
-  <si>
-    <t>e_JP158*</t>
-  </si>
-  <si>
-    <t>p_JP121</t>
-  </si>
-  <si>
-    <t>e_JP121*</t>
-  </si>
-  <si>
-    <t>p_JP124</t>
-  </si>
-  <si>
-    <t>e_JP124*</t>
-  </si>
-  <si>
-    <t>p_JP248</t>
-  </si>
-  <si>
-    <t>e_JP248*</t>
-  </si>
-  <si>
-    <t>p_JP76</t>
-  </si>
-  <si>
-    <t>e_JP76*</t>
-  </si>
-  <si>
-    <t>p_JP155</t>
-  </si>
-  <si>
-    <t>e_JP155*</t>
-  </si>
-  <si>
-    <t>p_JP219</t>
-  </si>
-  <si>
-    <t>e_JP219*</t>
-  </si>
-  <si>
-    <t>p_JP296</t>
-  </si>
-  <si>
-    <t>e_JP296*</t>
-  </si>
-  <si>
-    <t>p_JP74</t>
-  </si>
-  <si>
-    <t>e_JP74*</t>
-  </si>
-  <si>
-    <t>p_JP137</t>
-  </si>
-  <si>
-    <t>e_JP137*</t>
-  </si>
-  <si>
-    <t>p_JP50</t>
-  </si>
-  <si>
-    <t>e_JP50*</t>
-  </si>
-  <si>
-    <t>p_JP49</t>
-  </si>
-  <si>
-    <t>e_JP49*</t>
-  </si>
-  <si>
-    <t>p_JP249</t>
-  </si>
-  <si>
-    <t>e_JP249*</t>
-  </si>
-  <si>
-    <t>p_JP175</t>
-  </si>
-  <si>
-    <t>e_JP175*</t>
-  </si>
-  <si>
-    <t>p_JP306</t>
-  </si>
-  <si>
-    <t>e_JP306*</t>
-  </si>
-  <si>
-    <t>p_JP25</t>
-  </si>
-  <si>
-    <t>e_JP25*</t>
-  </si>
-  <si>
-    <t>p_JP101</t>
-  </si>
-  <si>
-    <t>e_JP101*</t>
-  </si>
-  <si>
-    <t>p_JP100</t>
-  </si>
-  <si>
-    <t>e_JP100*</t>
-  </si>
-  <si>
-    <t>p_JP103</t>
-  </si>
-  <si>
-    <t>e_JP103*</t>
-  </si>
-  <si>
-    <t>p_JP111</t>
-  </si>
-  <si>
-    <t>e_JP111*</t>
-  </si>
-  <si>
-    <t>p_JP109</t>
-  </si>
-  <si>
-    <t>e_JP109*</t>
-  </si>
-  <si>
-    <t>p_JP108</t>
-  </si>
-  <si>
-    <t>e_JP108*</t>
-  </si>
-  <si>
-    <t>p_JP107</t>
-  </si>
-  <si>
-    <t>e_JP107*</t>
-  </si>
-  <si>
-    <t>p_JP110</t>
-  </si>
-  <si>
-    <t>e_JP110*</t>
-  </si>
-  <si>
-    <t>p_JP120</t>
-  </si>
-  <si>
-    <t>e_JP120*</t>
-  </si>
-  <si>
-    <t>p_JP73</t>
-  </si>
-  <si>
-    <t>e_JP73*</t>
-  </si>
-  <si>
-    <t>p_w179863079</t>
-  </si>
-  <si>
-    <t>e_w179863079*</t>
-  </si>
-  <si>
-    <t>p_w801582512</t>
-  </si>
-  <si>
-    <t>e_w801582512*</t>
-  </si>
-  <si>
-    <t>p_JP5</t>
-  </si>
-  <si>
-    <t>e_JP5*</t>
-  </si>
-  <si>
-    <t>p_JP1</t>
-  </si>
-  <si>
-    <t>e_JP1*</t>
-  </si>
-  <si>
-    <t>p_JP2</t>
-  </si>
-  <si>
-    <t>e_JP2*</t>
-  </si>
-  <si>
-    <t>p_JP8</t>
-  </si>
-  <si>
-    <t>e_JP8*</t>
-  </si>
-  <si>
-    <t>p_JP7</t>
-  </si>
-  <si>
-    <t>e_JP7*</t>
-  </si>
-  <si>
-    <t>p_JP6</t>
-  </si>
-  <si>
-    <t>e_JP6*</t>
-  </si>
-  <si>
-    <t>p_JP4</t>
-  </si>
-  <si>
-    <t>e_JP4*</t>
-  </si>
-  <si>
-    <t>p_JP3</t>
-  </si>
-  <si>
-    <t>e_JP3*</t>
-  </si>
-  <si>
-    <t>rez_spv_001</t>
-  </si>
-  <si>
-    <t>elc_spv_001</t>
-  </si>
-  <si>
-    <t>rez_spv_002</t>
-  </si>
-  <si>
-    <t>elc_spv_002</t>
-  </si>
-  <si>
-    <t>rez_spv_003</t>
-  </si>
-  <si>
-    <t>elc_spv_003</t>
-  </si>
-  <si>
-    <t>rez_spv_004</t>
-  </si>
-  <si>
-    <t>elc_spv_004</t>
-  </si>
-  <si>
-    <t>rez_spv_005</t>
-  </si>
-  <si>
-    <t>elc_spv_005</t>
-  </si>
-  <si>
-    <t>rez_spv_006</t>
-  </si>
-  <si>
-    <t>elc_spv_006</t>
-  </si>
-  <si>
-    <t>rez_spv_007</t>
-  </si>
-  <si>
-    <t>elc_spv_007</t>
-  </si>
-  <si>
-    <t>rez_spv_008</t>
-  </si>
-  <si>
-    <t>elc_spv_008</t>
-  </si>
-  <si>
-    <t>rez_spv_009</t>
-  </si>
-  <si>
-    <t>elc_spv_009</t>
-  </si>
-  <si>
-    <t>rez_spv_010</t>
-  </si>
-  <si>
-    <t>elc_spv_010</t>
-  </si>
-  <si>
-    <t>rez_spv_011</t>
-  </si>
-  <si>
-    <t>elc_spv_011</t>
-  </si>
-  <si>
-    <t>rez_spv_012</t>
-  </si>
-  <si>
-    <t>elc_spv_012</t>
-  </si>
-  <si>
-    <t>rez_spv_013</t>
-  </si>
-  <si>
-    <t>elc_spv_013</t>
-  </si>
-  <si>
-    <t>rez_spv_014</t>
-  </si>
-  <si>
-    <t>elc_spv_014</t>
-  </si>
-  <si>
-    <t>rez_spv_015</t>
-  </si>
-  <si>
-    <t>elc_spv_015</t>
-  </si>
-  <si>
-    <t>rez_spv_016</t>
-  </si>
-  <si>
-    <t>elc_spv_016</t>
-  </si>
-  <si>
-    <t>rez_spv_017</t>
-  </si>
-  <si>
-    <t>elc_spv_017</t>
-  </si>
-  <si>
-    <t>rez_spv_018</t>
-  </si>
-  <si>
-    <t>elc_spv_018</t>
-  </si>
-  <si>
-    <t>rez_spv_019</t>
-  </si>
-  <si>
-    <t>elc_spv_019</t>
-  </si>
-  <si>
-    <t>rez_spv_020</t>
-  </si>
-  <si>
-    <t>elc_spv_020</t>
-  </si>
-  <si>
-    <t>rez_spv_021</t>
-  </si>
-  <si>
-    <t>elc_spv_021</t>
-  </si>
-  <si>
-    <t>rez_spv_022</t>
-  </si>
-  <si>
-    <t>elc_spv_022</t>
-  </si>
-  <si>
-    <t>rez_spv_023</t>
-  </si>
-  <si>
-    <t>elc_spv_023</t>
-  </si>
-  <si>
-    <t>rez_spv_024</t>
-  </si>
-  <si>
-    <t>elc_spv_024</t>
-  </si>
-  <si>
-    <t>rez_spv_025</t>
-  </si>
-  <si>
-    <t>elc_spv_025</t>
-  </si>
-  <si>
-    <t>rez_spv_026</t>
-  </si>
-  <si>
-    <t>elc_spv_026</t>
-  </si>
-  <si>
-    <t>rez_spv_027</t>
-  </si>
-  <si>
-    <t>elc_spv_027</t>
-  </si>
-  <si>
-    <t>rez_spv_028</t>
-  </si>
-  <si>
-    <t>elc_spv_028</t>
-  </si>
-  <si>
-    <t>rez_spv_029</t>
-  </si>
-  <si>
-    <t>elc_spv_029</t>
-  </si>
-  <si>
-    <t>rez_spv_030</t>
-  </si>
-  <si>
-    <t>elc_spv_030</t>
-  </si>
-  <si>
-    <t>rez_won_001</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>rez_won_002</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>rez_won_003</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>rez_won_004</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>rez_won_005</t>
-  </si>
-  <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>rez_won_006</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>rez_won_007</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>rez_won_008</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>rez_won_009</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>rez_won_010</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>rez_won_011</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>rez_won_012</t>
-  </si>
-  <si>
-    <t>elc_won_012</t>
-  </si>
-  <si>
-    <t>rez_won_013</t>
-  </si>
-  <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>rez_won_014</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>rez_won_015</t>
-  </si>
-  <si>
-    <t>elc_won_015</t>
-  </si>
-  <si>
-    <t>rez_won_016</t>
-  </si>
-  <si>
-    <t>elc_won_016</t>
-  </si>
-  <si>
-    <t>rez_won_017</t>
-  </si>
-  <si>
-    <t>elc_won_017</t>
-  </si>
-  <si>
-    <t>rez_won_018</t>
-  </si>
-  <si>
-    <t>elc_won_018</t>
-  </si>
-  <si>
-    <t>rez_won_019</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>rez_won_020</t>
-  </si>
-  <si>
-    <t>elc_won_020</t>
-  </si>
-  <si>
-    <t>rez_won_021</t>
-  </si>
-  <si>
-    <t>elc_won_021</t>
-  </si>
-  <si>
-    <t>rez_won_022</t>
-  </si>
-  <si>
-    <t>elc_won_022</t>
-  </si>
-  <si>
-    <t>rez_won_023</t>
-  </si>
-  <si>
-    <t>elc_won_023</t>
-  </si>
-  <si>
-    <t>rez_won_024</t>
-  </si>
-  <si>
-    <t>elc_won_024</t>
-  </si>
-  <si>
-    <t>rez_won_025</t>
-  </si>
-  <si>
-    <t>elc_won_025</t>
-  </si>
-  <si>
-    <t>rez_won_026</t>
-  </si>
-  <si>
-    <t>elc_won_026</t>
-  </si>
-  <si>
-    <t>rez_won_027</t>
-  </si>
-  <si>
-    <t>elc_won_027</t>
-  </si>
-  <si>
-    <t>rez_won_028</t>
-  </si>
-  <si>
-    <t>elc_won_028</t>
-  </si>
-  <si>
-    <t>rez_won_029</t>
-  </si>
-  <si>
-    <t>elc_won_029</t>
-  </si>
-  <si>
-    <t>rez_won_030</t>
-  </si>
-  <si>
-    <t>elc_won_030</t>
-  </si>
-  <si>
-    <t>rez_won_031</t>
-  </si>
-  <si>
-    <t>elc_won_031</t>
-  </si>
-  <si>
-    <t>rez_wof_001</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>rez_wof_002</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
-    <t>rez_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>rez_wof_004</t>
-  </si>
-  <si>
-    <t>elc_wof_004</t>
-  </si>
-  <si>
-    <t>rez_wof_005</t>
-  </si>
-  <si>
-    <t>elc_wof_005</t>
-  </si>
-  <si>
-    <t>rez_wof_006</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>rez_wof_007</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>rez_wof_008</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>rez_wof_009</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>rez_wof_010</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
-  </si>
-  <si>
-    <t>rez_wof_011</t>
-  </si>
-  <si>
-    <t>elc_wof_011</t>
-  </si>
-  <si>
-    <t>rez_wof_012</t>
-  </si>
-  <si>
-    <t>elc_wof_012</t>
-  </si>
-  <si>
-    <t>rez_wof_013</t>
-  </si>
-  <si>
-    <t>elc_wof_013</t>
-  </si>
-  <si>
-    <t>rez_wof_014</t>
-  </si>
-  <si>
-    <t>elc_wof_014</t>
-  </si>
-  <si>
-    <t>rez_wof_015</t>
-  </si>
-  <si>
-    <t>elc_wof_015</t>
-  </si>
-  <si>
-    <t>rez_wof_016</t>
-  </si>
-  <si>
-    <t>elc_wof_016</t>
-  </si>
-  <si>
-    <t>rez_wof_017</t>
-  </si>
-  <si>
-    <t>elc_wof_017</t>
-  </si>
-  <si>
-    <t>rez_wof_018</t>
-  </si>
-  <si>
-    <t>elc_wof_018</t>
-  </si>
-  <si>
-    <t>rez_wof_019</t>
-  </si>
-  <si>
-    <t>elc_wof_019</t>
-  </si>
-  <si>
-    <t>rez_wof_020</t>
-  </si>
-  <si>
-    <t>elc_wof_020</t>
-  </si>
-  <si>
-    <t>rez_wof_021</t>
-  </si>
-  <si>
-    <t>elc_wof_021</t>
-  </si>
-  <si>
-    <t>rez_wof_022</t>
-  </si>
-  <si>
-    <t>elc_wof_022</t>
-  </si>
-  <si>
-    <t>rez_wof_023</t>
-  </si>
-  <si>
-    <t>elc_wof_023</t>
-  </si>
-  <si>
-    <t>rez_wof_024</t>
-  </si>
-  <si>
-    <t>elc_wof_024</t>
-  </si>
-  <si>
-    <t>rez_wof_025</t>
-  </si>
-  <si>
-    <t>elc_wof_025</t>
-  </si>
-  <si>
-    <t>rez_wof_026</t>
-  </si>
-  <si>
-    <t>elc_wof_026</t>
-  </si>
-  <si>
-    <t>rez_wof_027</t>
-  </si>
-  <si>
-    <t>elc_wof_027</t>
-  </si>
-  <si>
-    <t>rez_wof_028</t>
-  </si>
-  <si>
-    <t>elc_wof_028</t>
-  </si>
-  <si>
-    <t>rez_wof_029</t>
-  </si>
-  <si>
-    <t>elc_wof_029</t>
-  </si>
-  <si>
-    <t>rez_wof_030</t>
-  </si>
-  <si>
-    <t>elc_wof_030</t>
-  </si>
-  <si>
-    <t>rez_wof_031</t>
-  </si>
-  <si>
-    <t>elc_wof_031</t>
-  </si>
-  <si>
-    <t>rez_wof_032</t>
-  </si>
-  <si>
-    <t>elc_wof_032</t>
-  </si>
-  <si>
-    <t>rez_wof_033</t>
-  </si>
-  <si>
-    <t>elc_wof_033</t>
-  </si>
-  <si>
-    <t>rez_wof_034</t>
-  </si>
-  <si>
-    <t>elc_wof_034</t>
-  </si>
-  <si>
-    <t>rez_wof_035</t>
-  </si>
-  <si>
-    <t>elc_wof_035</t>
-  </si>
-  <si>
-    <t>rez_wof_036</t>
-  </si>
-  <si>
-    <t>elc_wof_036</t>
-  </si>
-  <si>
-    <t>rez_wof_037</t>
-  </si>
-  <si>
-    <t>elc_wof_037</t>
-  </si>
-  <si>
-    <t>rez_wof_038</t>
-  </si>
-  <si>
-    <t>elc_wof_038</t>
-  </si>
-  <si>
-    <t>rez_wof_039</t>
-  </si>
-  <si>
-    <t>elc_wof_039</t>
-  </si>
-  <si>
-    <t>rez_wof_040</t>
-  </si>
-  <si>
-    <t>elc_wof_040</t>
-  </si>
-  <si>
-    <t>rez_wof_041</t>
-  </si>
-  <si>
-    <t>elc_wof_041</t>
-  </si>
-  <si>
-    <t>rez_wof_042</t>
-  </si>
-  <si>
-    <t>elc_wof_042</t>
-  </si>
-  <si>
-    <t>rez_wof_043</t>
-  </si>
-  <si>
-    <t>elc_wof_043</t>
-  </si>
-  <si>
-    <t>rez_wof_044</t>
-  </si>
-  <si>
-    <t>elc_wof_044</t>
+    <t>p_w87538349-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w87538349-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w102958903-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w102958903-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w104173570-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w104173570-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w104391636-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w104391636-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w104530060-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w104530060-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w105298089-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w105298089-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w106076988-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w106076988-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w106309481-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w106309481-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w109834508-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w109834508-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w109850439-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w109850439-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w110682956-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w110682956-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w116559939-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w116559939-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w128581912-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w128581912-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w132913106-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w132913106-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w133641619-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w133641619-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w133644487-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w133644487-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w142662111-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w142662111-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w145079972-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w145079972-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w149843487-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w149843487-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w150035494-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w150035494-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w150065045-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w150065045-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w151379730-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w151379730-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w156208858-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w156208858-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w161727149-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w161727149-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w161870227-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w161870227-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w161946849-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w161946849-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w168727982-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w168727982-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w168839127-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w168839127-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w168857610-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w168857610-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w169031921-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w169031921-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w169031998-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w169031998-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w169122898-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w169122898-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w169249243-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w169249243-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w256682313-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w256682313-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w169359724-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w169359724-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w169963227-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w169963227-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170247312-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170247312-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170366035-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170366035-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170537514-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170537514-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170568495-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170568495-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170589736-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170589736-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170605907-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170605907-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170850727-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170850727-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w170974371-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w170974371-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w171066843-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w171066843-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w172144358-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w172144358-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w172601929-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w172601929-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w172907196-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w172907196-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w174636874-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w174636874-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w185029969-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w185029969-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w186510275-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w186510275-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w187988970-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w187988970-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w190769051-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w190769051-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w193544791-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w193544791-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w195615141-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w195615141-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w201293312-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w201293312-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w204258596-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w204258596-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w209429410-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w209429410-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w209726348-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w209726348-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w210090094-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w210090094-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w211412000-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w211412000-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w215451416-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w215451416-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w216502300-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w216502300-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w216778426-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w216778426-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w216953915-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w216953915-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w216956620-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w216956620-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w241822621-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w241822621-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w241822623-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w241822623-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w241822631-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w241822631-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w241828221-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w241828221-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w242103481-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w242103481-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w242103532-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w242103532-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w242253500-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w242253500-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w250540807-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w250540807-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w253566674-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w253566674-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w291678103-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w291678103-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w307942220-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w307942220-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w315434358-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w315434358-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w315461259-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w315461259-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w315461272-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w315461272-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w315618377-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w315618377-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w315662839-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w315662839-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w317416612-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w317416612-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w317511904-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w317511904-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w320438391-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w320438391-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w405626236-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w405626236-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w421647841-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w421647841-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w459476442-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w459476442-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w505170104-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w505170104-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w659138214-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w659138214-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w714627759-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w714627759-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w722673849-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w722673849-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w785319805-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w785319805-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w832823487-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w832823487-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w901872431-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w901872431-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w901872439-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w901872439-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w1029010255-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w1029010255-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w975217734-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w975217734-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w1028554758-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w1028554758-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w1030329139-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w1030329139-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w1037299172-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w1037299172-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w1037516198-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w1037516198-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w1038584990-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w1038584990-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_r2269992-500_JPN</t>
+  </si>
+  <si>
+    <t>e_r2269992-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_r11529219-500_JPN</t>
+  </si>
+  <si>
+    <t>e_r11529219-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_r11529637-500_JPN</t>
+  </si>
+  <si>
+    <t>e_r11529637-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_r13768299-500_JPN</t>
+  </si>
+  <si>
+    <t>e_r13768299-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_r15580570-500_JPN</t>
+  </si>
+  <si>
+    <t>e_r15580570-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_r17013811-500_JPN</t>
+  </si>
+  <si>
+    <t>e_r17013811-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP21-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP21-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP36-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP36-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w66098469-1000_JPN</t>
+  </si>
+  <si>
+    <t>e_w66098469-1000_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP28-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP28-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w253566674-1000_JPN</t>
+  </si>
+  <si>
+    <t>e_w253566674-1000_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP60-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP60-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP23-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP23-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP95-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP95-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP191-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP191-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP116-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP116-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP156-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP156-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP141-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP141-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP122-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP122-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP178-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP178-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP117-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP117-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP132-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP132-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP269-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP269-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP19-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP19-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP267-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP267-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP102-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP102-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP112-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP112-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP106-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP106-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP96-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP96-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP9-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP9-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP292-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP292-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP294-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP294-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP41-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP41-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP29-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP29-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP37-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP37-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP218-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP218-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w242253537-500_JPN</t>
+  </si>
+  <si>
+    <t>e_w242253537-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP10-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP10-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP57-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP57-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP30-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP30-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP34-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP34-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP118-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP118-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP119-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP119-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP135-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP135-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP158-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP158-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP121-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP121-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP124-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP124-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP248-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP248-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP76-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP76-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP155-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP155-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP219-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP219-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP296-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP296-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP74-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP74-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP137-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP137-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP50-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP50-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP49-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP49-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP249-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP249-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP175-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP175-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP306-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP306-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP25-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP25-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP101-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP101-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP100-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP100-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP103-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP103-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP111-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP111-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP109-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP109-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP108-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP108-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP107-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP107-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP110-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP110-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_w250540807-1000_JPN</t>
+  </si>
+  <si>
+    <t>e_w250540807-1000_JPN*</t>
+  </si>
+  <si>
+    <t>p_w150035494-1000_JPN</t>
+  </si>
+  <si>
+    <t>e_w150035494-1000_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP120-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP120-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP73-500_JPN</t>
+  </si>
+  <si>
+    <t>e_JP73-500_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP28-1000_JPN</t>
+  </si>
+  <si>
+    <t>e_JP28-1000_JPN*</t>
+  </si>
+  <si>
+    <t>p_w179863079-275_JPN</t>
+  </si>
+  <si>
+    <t>e_w179863079-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_w801582512-275_JPN</t>
+  </si>
+  <si>
+    <t>e_w801582512-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP5-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP5-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP1-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP1-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP2-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP2-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP8-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP8-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP7-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP7-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP6-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP6-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP4-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP4-275_JPN*</t>
+  </si>
+  <si>
+    <t>p_JP3-275_JPN</t>
+  </si>
+  <si>
+    <t>e_JP3-275_JPN*</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_001</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_001</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_002</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_002</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_003</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_003</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_004</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_004</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_005</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_005</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_006</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_006</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_007</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_007</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_008</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_008</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_009</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_009</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_010</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_010</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_011</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_011</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_012</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_012</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_013</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_013</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_014</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_014</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_015</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_015</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_016</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_016</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_017</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_017</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_018</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_018</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_019</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_019</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_020</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_020</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_021</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_021</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_022</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_022</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_023</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_023</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_024</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_024</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_025</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_025</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_026</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_026</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_027</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_027</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_028</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_028</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_029</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_029</t>
+  </si>
+  <si>
+    <t>rez_spv_JPN_030</t>
+  </si>
+  <si>
+    <t>elc_spv_JPN_030</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_001</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_001</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_002</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_002</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_003</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_003</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_004</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_004</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_005</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_005</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_006</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_006</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_007</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_007</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_008</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_008</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_009</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_009</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_010</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_010</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_011</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_011</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_012</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_012</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_013</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_013</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_014</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_014</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_015</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_015</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_016</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_016</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_017</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_017</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_018</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_018</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_019</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_019</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_020</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_020</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_021</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_021</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_022</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_022</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_023</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_023</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_024</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_024</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_025</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_025</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_026</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_026</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_027</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_027</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_028</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_028</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_029</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_029</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_030</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_030</t>
+  </si>
+  <si>
+    <t>rez_won_JPN_031</t>
+  </si>
+  <si>
+    <t>elc_won_JPN_031</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_001</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_001</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_002</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_002</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_003</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_003</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_004</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_004</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_005</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_005</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_006</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_006</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_007</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_007</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_008</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_008</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_009</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_009</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_010</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_010</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_011</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_011</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_012</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_012</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_013</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_013</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_014</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_014</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_015</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_015</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_016</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_016</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_017</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_017</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_018</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_018</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_019</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_019</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_020</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_020</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_021</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_021</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_022</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_022</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_023</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_023</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_024</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_024</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_025</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_025</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_026</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_026</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_027</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_027</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_028</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_028</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_029</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_029</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_030</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_030</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_031</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_031</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_032</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_032</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_033</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_033</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_034</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_034</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_035</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_035</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_036</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_036</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_037</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_037</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_038</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_038</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_039</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_039</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_040</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_040</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_041</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_041</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_042</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_042</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_043</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_043</t>
+  </si>
+  <si>
+    <t>rez_wof_JPN_044</t>
+  </si>
+  <si>
+    <t>elc_wof_JPN_044</t>
   </si>
 </sst>
 </file>
@@ -2168,9 +2198,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2208,7 +2238,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2314,7 +2344,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2456,7 +2486,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2909,8 +2939,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89898591-2AEA-456B-83A2-A8912B3A7DE3}">
-  <dimension ref="B9:E297"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62FE220E-2815-491A-A9C7-90C6B778A99B}">
+  <dimension ref="B9:E302"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -6947,6 +6977,76 @@
         <v>677</v>
       </c>
       <c r="E297" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="298" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B298" t="s">
+        <v>678</v>
+      </c>
+      <c r="C298" t="s">
+        <v>679</v>
+      </c>
+      <c r="D298" t="s">
+        <v>679</v>
+      </c>
+      <c r="E298" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="299" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B299" t="s">
+        <v>680</v>
+      </c>
+      <c r="C299" t="s">
+        <v>681</v>
+      </c>
+      <c r="D299" t="s">
+        <v>681</v>
+      </c>
+      <c r="E299" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="300" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B300" t="s">
+        <v>682</v>
+      </c>
+      <c r="C300" t="s">
+        <v>683</v>
+      </c>
+      <c r="D300" t="s">
+        <v>683</v>
+      </c>
+      <c r="E300" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="301" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B301" t="s">
+        <v>684</v>
+      </c>
+      <c r="C301" t="s">
+        <v>685</v>
+      </c>
+      <c r="D301" t="s">
+        <v>685</v>
+      </c>
+      <c r="E301" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="302" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B302" t="s">
+        <v>686</v>
+      </c>
+      <c r="C302" t="s">
+        <v>687</v>
+      </c>
+      <c r="D302" t="s">
+        <v>687</v>
+      </c>
+      <c r="E302" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>